<commit_message>
Update tool, tests and docs
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/edge-cases.xlsx
+++ b/tests/fixtures/edge-cases.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -459,18 +459,42 @@
         <v>46090.5</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Barcode</v>
+      </c>
+      <c r="B8">
+        <v>9780306406157</v>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="B9">
+        <v>447123456789</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Ratio</v>
+      </c>
+      <c r="B10">
+        <v>0.30000000000000004</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v/>
       </c>
     </row>
-    <row r="10"/>
+    <row r="13"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>